<commit_message>
Complete ORCS enrichment synthesis milestone
</commit_message>
<xml_diff>
--- a/data/templates/BioStudies-ArrayExpress-Enrichment.xlsx
+++ b/data/templates/BioStudies-ArrayExpress-Enrichment.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Studies" sheetId="1" r:id="R79517a6828204e8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repository citations" sheetId="2" r:id="Rc41235c5f33e4ed1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protocols" sheetId="3" r:id="R57a6dd07522d4211"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sample metadata" sheetId="4" r:id="R15fa3ffb93394b14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assay metadata" sheetId="5" r:id="R11479c90d5c0452e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="File listings" sheetId="6" r:id="Rf0ddcb6f457340d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SDRF metadata" sheetId="7" r:id="R31a002c967d14db6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IDF metadata" sheetId="8" r:id="R22be92b16ea64d27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Studies" sheetId="1" r:id="R9eb66d726f79499e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repository citations" sheetId="2" r:id="R7a7bbb256bce4bf1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protocols" sheetId="3" r:id="R9714388a6a20409d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sample metadata" sheetId="4" r:id="Rb56542ea5ec74d83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assay metadata" sheetId="5" r:id="R63f24d45597448f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="File listings" sheetId="6" r:id="Rde1a7f23fc2f4d88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SDRF metadata" sheetId="7" r:id="Rabe9656acf994711"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IDF metadata" sheetId="8" r:id="R5bdc41a1fccd4b4f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20,6 +20,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="@"/>
+  </x:numFmts>
   <x:fonts count="2">
     <x:font>
       <x:sz val="11"/>
@@ -51,9 +54,21 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="2">
+  <x:cellXfs count="6">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -256,47 +271,47 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="22" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="22" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="22" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="52" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="25" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="25" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="25" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="25" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="80" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="25" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="25" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="1" t="str">
+    <x:row r="1" ht="46" customHeight="1">
+      <x:c r="A1" s="5" t="str">
         <x:v>Study accession</x:v>
       </x:c>
-      <x:c r="B1" s="1" t="str">
+      <x:c r="B1" s="5" t="str">
         <x:v>PMID</x:v>
       </x:c>
-      <x:c r="C1" s="1" t="str">
+      <x:c r="C1" s="5" t="str">
         <x:v>Study title</x:v>
       </x:c>
-      <x:c r="D1" s="1" t="str">
+      <x:c r="D1" s="5" t="str">
         <x:v>Organism</x:v>
       </x:c>
-      <x:c r="E1" s="1" t="str">
+      <x:c r="E1" s="5" t="str">
         <x:v>Study type</x:v>
       </x:c>
-      <x:c r="F1" s="1" t="str">
+      <x:c r="F1" s="5" t="str">
         <x:v>Samples reported</x:v>
       </x:c>
-      <x:c r="G1" s="1" t="str">
+      <x:c r="G1" s="5" t="str">
         <x:v>Assays reported</x:v>
       </x:c>
-      <x:c r="H1" s="1" t="str">
+      <x:c r="H1" s="5" t="str">
         <x:v>Study description</x:v>
       </x:c>
-      <x:c r="I1" s="1" t="str">
+      <x:c r="I1" s="5" t="str">
         <x:v>Publication association</x:v>
       </x:c>
-      <x:c r="J1" s="1" t="str">
+      <x:c r="J1" s="5" t="str">
         <x:v>Source URL</x:v>
       </x:c>
     </x:row>
@@ -309,35 +324,35 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="52" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="25" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="25" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="52" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="25" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="25" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="1" t="str">
+    <x:row r="1" ht="46" customHeight="1">
+      <x:c r="A1" s="5" t="str">
         <x:v>Study accession</x:v>
       </x:c>
-      <x:c r="B1" s="1" t="str">
+      <x:c r="B1" s="5" t="str">
         <x:v>Native citation title</x:v>
       </x:c>
-      <x:c r="C1" s="1" t="str">
+      <x:c r="C1" s="5" t="str">
         <x:v>Native DOI</x:v>
       </x:c>
-      <x:c r="D1" s="1" t="str">
+      <x:c r="D1" s="5" t="str">
         <x:v>Native PMID</x:v>
       </x:c>
-      <x:c r="E1" s="1" t="str">
+      <x:c r="E1" s="5" t="str">
         <x:v>Native authors</x:v>
       </x:c>
-      <x:c r="F1" s="1" t="str">
+      <x:c r="F1" s="5" t="str">
         <x:v>Native status</x:v>
       </x:c>
-      <x:c r="G1" s="1" t="str">
+      <x:c r="G1" s="5" t="str">
         <x:v>Source URL</x:v>
       </x:c>
     </x:row>
@@ -350,28 +365,40 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="80" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="80" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="25" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="25" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="25" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="25" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="25" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="1" t="str">
+    <x:row r="1" ht="46" customHeight="1">
+      <x:c r="A1" s="5" t="str">
         <x:v>Study accession</x:v>
       </x:c>
-      <x:c r="B1" s="1" t="str">
+      <x:c r="B1" s="5" t="str">
         <x:v>Native protocol ID</x:v>
       </x:c>
-      <x:c r="C1" s="1" t="str">
-        <x:v>Field</x:v>
-      </x:c>
-      <x:c r="D1" s="1" t="str">
-        <x:v>Original value</x:v>
-      </x:c>
-      <x:c r="E1" s="1" t="str">
-        <x:v>Value state</x:v>
+      <x:c r="C1" s="5" t="str">
+        <x:v>Description</x:v>
+      </x:c>
+      <x:c r="D1" s="5" t="str">
+        <x:v>Hardware</x:v>
+      </x:c>
+      <x:c r="E1" s="5" t="str">
+        <x:v>Name</x:v>
+      </x:c>
+      <x:c r="F1" s="5" t="str">
+        <x:v>Parameters</x:v>
+      </x:c>
+      <x:c r="G1" s="5" t="str">
+        <x:v>Software</x:v>
+      </x:c>
+      <x:c r="H1" s="5" t="str">
+        <x:v>Type</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -383,32 +410,200 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="25" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="25" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="25" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="25" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="25" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="25" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="25" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="25" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="25" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="25" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="25" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="25" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="25" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="25" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="25" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="25" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="25" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="25" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="25" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="25" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="25" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="25" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="25" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="25" hidden="0" customWidth="1"/>
+    <x:col min="27" max="27" width="25" hidden="0" customWidth="1"/>
+    <x:col min="28" max="28" width="25" hidden="0" customWidth="1"/>
+    <x:col min="29" max="29" width="25" hidden="0" customWidth="1"/>
+    <x:col min="30" max="30" width="25" hidden="0" customWidth="1"/>
+    <x:col min="31" max="31" width="25" hidden="0" customWidth="1"/>
+    <x:col min="32" max="32" width="25" hidden="0" customWidth="1"/>
+    <x:col min="33" max="33" width="25" hidden="0" customWidth="1"/>
+    <x:col min="34" max="34" width="25" hidden="0" customWidth="1"/>
+    <x:col min="35" max="35" width="25" hidden="0" customWidth="1"/>
+    <x:col min="36" max="36" width="25" hidden="0" customWidth="1"/>
+    <x:col min="37" max="37" width="25" hidden="0" customWidth="1"/>
+    <x:col min="38" max="38" width="25" hidden="0" customWidth="1"/>
+    <x:col min="39" max="39" width="25" hidden="0" customWidth="1"/>
+    <x:col min="40" max="40" width="25" hidden="0" customWidth="1"/>
+    <x:col min="41" max="41" width="25" hidden="0" customWidth="1"/>
+    <x:col min="42" max="42" width="25" hidden="0" customWidth="1"/>
+    <x:col min="43" max="43" width="25" hidden="0" customWidth="1"/>
+    <x:col min="44" max="44" width="25" hidden="0" customWidth="1"/>
+    <x:col min="45" max="45" width="25" hidden="0" customWidth="1"/>
+    <x:col min="46" max="46" width="25" hidden="0" customWidth="1"/>
+    <x:col min="47" max="47" width="25" hidden="0" customWidth="1"/>
+    <x:col min="48" max="48" width="25" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="1" t="str">
+    <x:row r="1" ht="46" customHeight="1">
+      <x:c r="A1" s="5" t="str">
         <x:v>Study accession</x:v>
       </x:c>
-      <x:c r="B1" s="1" t="str">
+      <x:c r="B1" s="5" t="str">
+        <x:v>Native section ID</x:v>
+      </x:c>
+      <x:c r="C1" s="5" t="str">
         <x:v>Native section type</x:v>
       </x:c>
-      <x:c r="C1" s="1" t="str">
-        <x:v>Native section ID</x:v>
-      </x:c>
-      <x:c r="D1" s="1" t="str">
-        <x:v>Field</x:v>
-      </x:c>
-      <x:c r="E1" s="1" t="str">
-        <x:v>Original value</x:v>
-      </x:c>
-      <x:c r="F1" s="1" t="str">
-        <x:v>Value state</x:v>
+      <x:c r="D1" s="5" t="str">
+        <x:v>Age</x:v>
+      </x:c>
+      <x:c r="E1" s="5" t="str">
+        <x:v>Cell line</x:v>
+      </x:c>
+      <x:c r="F1" s="5" t="str">
+        <x:v>Cell type</x:v>
+      </x:c>
+      <x:c r="G1" s="5" t="str">
+        <x:v>Compound</x:v>
+      </x:c>
+      <x:c r="H1" s="5" t="str">
+        <x:v>Developmental stage</x:v>
+      </x:c>
+      <x:c r="I1" s="5" t="str">
+        <x:v>Disease</x:v>
+      </x:c>
+      <x:c r="J1" s="5" t="str">
+        <x:v>Dose</x:v>
+      </x:c>
+      <x:c r="K1" s="5" t="str">
+        <x:v>Experimental Designs</x:v>
+      </x:c>
+      <x:c r="L1" s="5" t="str">
+        <x:v>Experimental Factors</x:v>
+      </x:c>
+      <x:c r="M1" s="5" t="str">
+        <x:v>Gbm subtype</x:v>
+      </x:c>
+      <x:c r="N1" s="5" t="str">
+        <x:v>Genetic modification</x:v>
+      </x:c>
+      <x:c r="O1" s="5" t="str">
+        <x:v>Genotype</x:v>
+      </x:c>
+      <x:c r="P1" s="5" t="str">
+        <x:v>Infect</x:v>
+      </x:c>
+      <x:c r="Q1" s="5" t="str">
+        <x:v>Isolate</x:v>
+      </x:c>
+      <x:c r="R1" s="5" t="str">
+        <x:v>Material type</x:v>
+      </x:c>
+      <x:c r="S1" s="5" t="str">
+        <x:v>No. of Samples</x:v>
+      </x:c>
+      <x:c r="T1" s="5" t="str">
+        <x:v>Organism</x:v>
+      </x:c>
+      <x:c r="U1" s="5" t="str">
+        <x:v>Organism part</x:v>
+      </x:c>
+      <x:c r="V1" s="5" t="str">
+        <x:v>RNA interference</x:v>
+      </x:c>
+      <x:c r="W1" s="5" t="str">
+        <x:v>Rna interference</x:v>
+      </x:c>
+      <x:c r="X1" s="5" t="str">
+        <x:v>Sample count</x:v>
+      </x:c>
+      <x:c r="Y1" s="5" t="str">
+        <x:v>Sampling time point</x:v>
+      </x:c>
+      <x:c r="Z1" s="5" t="str">
+        <x:v>Sex</x:v>
+      </x:c>
+      <x:c r="AA1" s="5" t="str">
+        <x:v>Source</x:v>
+      </x:c>
+      <x:c r="AB1" s="5" t="str">
+        <x:v>Stimulus</x:v>
+      </x:c>
+      <x:c r="AC1" s="5" t="str">
+        <x:v>Strain</x:v>
+      </x:c>
+      <x:c r="AD1" s="5" t="str">
+        <x:v>Time</x:v>
+      </x:c>
+      <x:c r="AE1" s="5" t="str">
+        <x:v>age</x:v>
+      </x:c>
+      <x:c r="AF1" s="5" t="str">
+        <x:v>cell line</x:v>
+      </x:c>
+      <x:c r="AG1" s="5" t="str">
+        <x:v>cell type</x:v>
+      </x:c>
+      <x:c r="AH1" s="5" t="str">
+        <x:v>compound</x:v>
+      </x:c>
+      <x:c r="AI1" s="5" t="str">
+        <x:v>developmental stage</x:v>
+      </x:c>
+      <x:c r="AJ1" s="5" t="str">
+        <x:v>disease</x:v>
+      </x:c>
+      <x:c r="AK1" s="5" t="str">
+        <x:v>gbm subtype</x:v>
+      </x:c>
+      <x:c r="AL1" s="5" t="str">
+        <x:v>genetic modification</x:v>
+      </x:c>
+      <x:c r="AM1" s="5" t="str">
+        <x:v>genotype</x:v>
+      </x:c>
+      <x:c r="AN1" s="5" t="str">
+        <x:v>infect</x:v>
+      </x:c>
+      <x:c r="AO1" s="5" t="str">
+        <x:v>isolate</x:v>
+      </x:c>
+      <x:c r="AP1" s="5" t="str">
+        <x:v>material type</x:v>
+      </x:c>
+      <x:c r="AQ1" s="5" t="str">
+        <x:v>organism part</x:v>
+      </x:c>
+      <x:c r="AR1" s="5" t="str">
+        <x:v>sampling time point</x:v>
+      </x:c>
+      <x:c r="AS1" s="5" t="str">
+        <x:v>sex</x:v>
+      </x:c>
+      <x:c r="AT1" s="5" t="str">
+        <x:v>stimulus</x:v>
+      </x:c>
+      <x:c r="AU1" s="5" t="str">
+        <x:v>strain</x:v>
+      </x:c>
+      <x:c r="AV1" s="5" t="str">
+        <x:v>time</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -420,32 +615,32 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="25" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="25" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="25" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="25" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="1" t="str">
+    <x:row r="1" ht="46" customHeight="1">
+      <x:c r="A1" s="5" t="str">
         <x:v>Study accession</x:v>
       </x:c>
-      <x:c r="B1" s="1" t="str">
+      <x:c r="B1" s="5" t="str">
+        <x:v>Native section ID</x:v>
+      </x:c>
+      <x:c r="C1" s="5" t="str">
         <x:v>Native section type</x:v>
       </x:c>
-      <x:c r="C1" s="1" t="str">
-        <x:v>Native section ID</x:v>
-      </x:c>
-      <x:c r="D1" s="1" t="str">
-        <x:v>Field</x:v>
-      </x:c>
-      <x:c r="E1" s="1" t="str">
-        <x:v>Original value</x:v>
-      </x:c>
-      <x:c r="F1" s="1" t="str">
-        <x:v>Value state</x:v>
+      <x:c r="D1" s="5" t="str">
+        <x:v>Assay by Molecule</x:v>
+      </x:c>
+      <x:c r="E1" s="5" t="str">
+        <x:v>Assay count</x:v>
+      </x:c>
+      <x:c r="F1" s="5" t="str">
+        <x:v>Technology</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -457,35 +652,35 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="25" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="25" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="25" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="25" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="80" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="1" t="str">
+    <x:row r="1" ht="46" customHeight="1">
+      <x:c r="A1" s="5" t="str">
         <x:v>Study accession</x:v>
       </x:c>
-      <x:c r="B1" s="1" t="str">
+      <x:c r="B1" s="5" t="str">
         <x:v>Native section type</x:v>
       </x:c>
-      <x:c r="C1" s="1" t="str">
+      <x:c r="C1" s="5" t="str">
         <x:v>File path</x:v>
       </x:c>
-      <x:c r="D1" s="1" t="str">
+      <x:c r="D1" s="5" t="str">
         <x:v>Size (bytes)</x:v>
       </x:c>
-      <x:c r="E1" s="1" t="str">
+      <x:c r="E1" s="5" t="str">
         <x:v>Declared type</x:v>
       </x:c>
-      <x:c r="F1" s="1" t="str">
+      <x:c r="F1" s="5" t="str">
         <x:v>Format</x:v>
       </x:c>
-      <x:c r="G1" s="1" t="str">
+      <x:c r="G1" s="5" t="str">
         <x:v>Description</x:v>
       </x:c>
     </x:row>
@@ -498,35 +693,35 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="52" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="25" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="25" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="52" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="52" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="25" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="1" t="str">
+    <x:row r="1" ht="46" customHeight="1">
+      <x:c r="A1" s="5" t="str">
         <x:v>Study accession</x:v>
       </x:c>
-      <x:c r="B1" s="1" t="str">
+      <x:c r="B1" s="5" t="str">
         <x:v>Source name</x:v>
       </x:c>
-      <x:c r="C1" s="1" t="str">
+      <x:c r="C1" s="5" t="str">
         <x:v>Native data row</x:v>
       </x:c>
-      <x:c r="D1" s="1" t="str">
+      <x:c r="D1" s="5" t="str">
         <x:v>Native column</x:v>
       </x:c>
-      <x:c r="E1" s="1" t="str">
+      <x:c r="E1" s="5" t="str">
         <x:v>Native field</x:v>
       </x:c>
-      <x:c r="F1" s="1" t="str">
+      <x:c r="F1" s="5" t="str">
         <x:v>Original value</x:v>
       </x:c>
-      <x:c r="G1" s="1" t="str">
+      <x:c r="G1" s="5" t="str">
         <x:v>Part</x:v>
       </x:c>
     </x:row>
@@ -539,27 +734,27 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="25" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="52" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="52" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="1" t="str">
+    <x:row r="1" ht="46" customHeight="1">
+      <x:c r="A1" s="5" t="str">
         <x:v>Study accession</x:v>
       </x:c>
-      <x:c r="B1" s="1" t="str">
+      <x:c r="B1" s="5" t="str">
         <x:v>Native line</x:v>
       </x:c>
-      <x:c r="C1" s="1" t="str">
+      <x:c r="C1" s="5" t="str">
         <x:v>Native column</x:v>
       </x:c>
-      <x:c r="D1" s="1" t="str">
+      <x:c r="D1" s="5" t="str">
         <x:v>Native field</x:v>
       </x:c>
-      <x:c r="E1" s="1" t="str">
+      <x:c r="E1" s="5" t="str">
         <x:v>Original value</x:v>
       </x:c>
     </x:row>

</xml_diff>